<commit_message>
Polish dashboard formatting and interactive charts
</commit_message>
<xml_diff>
--- a/Wedding_Guest_Analytics_Dashboard.xlsx
+++ b/Wedding_Guest_Analytics_Dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/373b1d010945caec/Desktop/Projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{492472DB-7E8D-4C61-BA57-3FDEA99F323E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7351417A-4A69-45F8-A27F-D7A772048DC6}"/>
+  <xr:revisionPtr revIDLastSave="243" documentId="8_{492472DB-7E8D-4C61-BA57-3FDEA99F323E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BE1D6D9-E584-4C67-AF8B-CEFE3A50CB6F}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pivot Analysis" sheetId="6" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="173">
   <si>
     <t>Groom</t>
   </si>
@@ -572,9 +572,6 @@
   </si>
   <si>
     <t>Select a relationship category to filter the Interactive Attendance by Inviter chart. Other metrics display overall totals.</t>
-  </si>
-  <si>
-    <t>RSVP Acceptance Rate</t>
   </si>
 </sst>
 </file>
@@ -715,7 +712,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -724,6 +720,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2468,7 +2465,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.1196157961170884"/>
+          <c:y val="0.13059895833333335"/>
+          <c:w val="0.8284758069363467"/>
+          <c:h val="0.73833217136920382"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -4179,37 +4186,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -4254,11 +4230,8 @@
   <c:extLst>
     <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
       <c14:pivotOptions>
-        <c14:dropZoneFilter val="1"/>
         <c14:dropZoneCategories val="1"/>
         <c14:dropZoneData val="1"/>
-        <c14:dropZoneSeries val="1"/>
-        <c14:dropZonesVisible val="1"/>
       </c14:pivotOptions>
     </c:ext>
     <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
@@ -8816,15 +8789,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>12700</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>163830</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>55880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8853,16 +8826,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>44450</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>163830</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>31750</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>55880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8893,14 +8866,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>12700</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>163830</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>93980</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8929,16 +8902,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>374650</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>44450</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>163830</xdr:rowOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>93980</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8968,18 +8941,18 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1828800</xdr:colOff>
-      <xdr:row>68</xdr:row>
-      <xdr:rowOff>130175</xdr:rowOff>
+      <xdr:colOff>1841500</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="6" name="Relation">
@@ -9002,7 +8975,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -9012,8 +8985,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="0" y="11150600"/>
-              <a:ext cx="1828800" cy="2524125"/>
+              <a:off x="12700" y="9757833"/>
+              <a:ext cx="1828800" cy="2464859"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -10491,7 +10464,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E8BD8A31-A30B-4953-9CDE-F86F19F744AE}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E8BD8A31-A30B-4953-9CDE-F86F19F744AE}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -15210,24 +15183,28 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CA2B964-C8D8-4361-8628-BB39775E0555}">
-  <dimension ref="A1:H55"/>
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="45.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.36328125" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="42" customHeight="1">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="9" t="s">
@@ -15312,37 +15289,29 @@
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
     </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="11" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="31">
-      <c r="A13" s="16">
-        <f>COUNTIF(WeddingGuests[RSVP],"Y")/COUNTA(WeddingGuests[RSVP])</f>
-        <v>0.46825396825396826</v>
-      </c>
+    <row r="12" spans="1:8" ht="15.5">
+      <c r="A12" s="17" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="17" customHeight="1">
+      <c r="A13" s="20"/>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1">
-      <c r="A14" s="16"/>
-    </row>
-    <row r="15" spans="1:8" ht="15.5">
-      <c r="A15" s="18" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="15.5">
-      <c r="A34" s="17" t="s">
+      <c r="A14" s="20"/>
+    </row>
+    <row r="30" spans="1:1" ht="15.5">
+      <c r="A30" s="16" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="54" spans="1:1" ht="15.5">
-      <c r="A54" s="17" t="s">
+    <row r="48" spans="1:1" ht="15.5">
+      <c r="A48" s="16" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="55" spans="1:1">
-      <c r="A55" t="s">
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
         <v>172</v>
       </c>
     </row>
@@ -15351,11 +15320,12 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
       <x14:slicerList>
-        <x14:slicer r:id="rId2"/>
+        <x14:slicer r:id="rId3"/>
       </x14:slicerList>
     </ext>
   </extLst>

</xml_diff>